<commit_message>
Proyecto terminado (se procederá a mejorar caso de examen DIB TEC y luego conversion JAR ejecutable)
</commit_message>
<xml_diff>
--- a/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
+++ b/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
@@ -1,18 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr date1904="false"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sfer4\Desktop\AVANCES\RepositoriosLocales\0024_24072026_JAVA_MAVEN\0001-Proyecto-Maven-POI\ficherosGenerados\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4309837C-F5F5-45A0-8D06-4487E75372D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="EXAMEN" r:id="rId3" sheetId="1"/>
+    <sheet name="EXAMEN" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>ALUMNO:</t>
   </si>
@@ -77,16 +85,19 @@
     <t>Física y Química</t>
   </si>
   <si>
+    <t>Cinemática Vectorial</t>
+  </si>
+  <si>
+    <t>Cinemática Tiro Parabólico</t>
+  </si>
+  <si>
+    <t>Dinámica Cantidad Movimiento</t>
+  </si>
+  <si>
     <t>Cinemática MRU MRUA MCU MCUA</t>
   </si>
   <si>
-    <t>Cinemática Tiro Parabólico</t>
-  </si>
-  <si>
-    <t>Cinemática Vectorial</t>
-  </si>
-  <si>
-    <t>Jueves, dia 13 de Agosto del 2026</t>
+    <t>Sábado, dia 29 de Agosto del 2026</t>
   </si>
   <si>
     <t>A las: 16:00 horas</t>
@@ -98,61 +109,60 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
     </font>
     <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
     </font>
     <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
     </font>
     <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
     </font>
     <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
     </font>
     <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
     </font>
     <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
     </font>
   </fonts>
   <fills count="2">
@@ -160,7 +170,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="darkGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="3">
@@ -172,10 +182,22 @@
       <diagonal/>
     </border>
     <border>
-      <bottom style="thin"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
     <border>
-      <bottom style="thick"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -183,23 +205,36 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="twoCell">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -214,13 +249,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -237,7 +278,7 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -252,13 +293,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPr id="3" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -283,20 +330,26 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>3619500</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>628650</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3390900</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>771525</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPr id="4" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -304,7 +357,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3619500" cy="628650"/>
+          <a:ext cx="6524625" cy="1724025"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -321,20 +374,26 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>3619500</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>619125</xdr:rowOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>733425</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPr id="5" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -342,7 +401,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3619500" cy="619125"/>
+          <a:ext cx="6753225" cy="1685925"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -359,20 +418,26 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>3619500</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>409575</xdr:rowOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>933450</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPr id="6" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -380,7 +445,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3619500" cy="409575"/>
+          <a:ext cx="6753225" cy="1885950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -397,20 +462,26 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>3619500</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>914400</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3305175</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>523875</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPr id="7" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -418,7 +489,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3619500" cy="914400"/>
+          <a:ext cx="6438900" cy="1476375"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -435,20 +506,26 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>3619500</xdr:colOff>
-      <xdr:row>71</xdr:row>
-      <xdr:rowOff>457200</xdr:rowOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>333375</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPr id="8" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -456,7 +533,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3619500" cy="457200"/>
+          <a:ext cx="6753225" cy="1285875"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -473,20 +550,26 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>3619500</xdr:colOff>
-      <xdr:row>91</xdr:row>
-      <xdr:rowOff>514350</xdr:rowOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>457200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPr id="9" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -494,7 +577,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3619500" cy="514350"/>
+          <a:ext cx="6753225" cy="1409700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -506,109 +589,404 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H91"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.0" customWidth="true"/>
-    <col min="8" max="8" width="13.0" customWidth="true"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s" s="8">
+      <c r="F1" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="1">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="1">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="1">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s" s="0">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="1">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="1">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="s" s="1">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
@@ -617,7 +995,7 @@
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
@@ -626,7 +1004,7 @@
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
@@ -635,7 +1013,7 @@
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -645,43 +1023,43 @@
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
     </row>
-    <row r="19">
-      <c r="A19" t="s" s="2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="s" s="3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="s" s="4">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="s" s="5">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="s" s="6">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="s" s="7">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" s="7" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.76" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.76"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.76" bottom="0.76" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;CPRUEBA DE EVALUACION ARCES 3 FORMACION</oddHeader>
     <oddFooter>&amp;RPágina &amp;P de &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adicionados mensajes de advertencia al ejecutable JAR generado del proyecto
</commit_message>
<xml_diff>
--- a/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
+++ b/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="28">
   <si>
     <t>ALUMNO:</t>
   </si>
@@ -77,6 +77,18 @@
     <t>Dibujo Técnico</t>
   </si>
   <si>
+    <t>Sistema Diédrico</t>
+  </si>
+  <si>
+    <t>Sábado, dia 15 de Agosto del 2026</t>
+  </si>
+  <si>
+    <t>A las: 02:30 horas</t>
+  </si>
+  <si>
+    <t>CALIFICACIÓN</t>
+  </si>
+  <si>
     <t>Construcción de Formas Polígonales</t>
   </si>
   <si>
@@ -84,9 +96,6 @@
   </si>
   <si>
     <t>A las: 16:00 horas</t>
-  </si>
-  <si>
-    <t>CALIFICACIÓN</t>
   </si>
 </sst>
 </file>
@@ -94,13 +103,59 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="17">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -175,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
@@ -187,6 +242,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -405,6 +470,462 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3609975</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>4581525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6743700" cy="6867525"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3619500</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>3943350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6753225" cy="6229350"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3552825</xdr:colOff>
+      <xdr:row>114</xdr:row>
+      <xdr:rowOff>4133850</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6686550" cy="6419850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>152</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3619500</xdr:colOff>
+      <xdr:row>164</xdr:row>
+      <xdr:rowOff>3171825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6753225" cy="5457825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>202</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3524250</xdr:colOff>
+      <xdr:row>214</xdr:row>
+      <xdr:rowOff>4657725</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6657975" cy="6943725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>252</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3619500</xdr:colOff>
+      <xdr:row>264</xdr:row>
+      <xdr:rowOff>3105150</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6753225" cy="5391150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>147</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>149</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>197</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>199</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>247</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>249</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>297</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>299</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId18"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -429,23 +950,23 @@
   <dimension ref="A1:H252"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="15.0" customWidth="true"/>
-    <col min="8" max="8" width="13.0" customWidth="true"/>
+    <col min="1" max="1" customWidth="true" width="15.0"/>
+    <col min="8" max="8" customWidth="true" width="13.0"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="1">
+      <c r="A1" t="s" s="11">
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="F1" t="s" s="8">
+      <c r="F1" t="s" s="18">
         <v>24</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="1">
+      <c r="A2" t="s" s="11">
         <v>1</v>
       </c>
       <c r="B2" t="s" s="0">
@@ -453,7 +974,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="1">
+      <c r="A3" t="s" s="11">
         <v>2</v>
       </c>
       <c r="B3" t="s" s="0">
@@ -461,107 +982,116 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="1">
+      <c r="A4" t="s" s="11">
         <v>3</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="1">
+      <c r="A5" t="s" s="11">
         <v>4</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="1">
+      <c r="A6" t="s" s="11">
         <v>5</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="1">
+      <c r="A7" t="s" s="11">
         <v>6</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s" s="1">
+      <c r="A8" t="s" s="11">
         <v>7</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s" s="1">
+      <c r="A9" t="s" s="11">
         <v>8</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s" s="1">
+      <c r="A10" t="s" s="11">
         <v>9</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="s" s="1">
+      <c r="A11" t="s" s="11">
         <v>10</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s" s="1">
+      <c r="A12" t="s" s="11">
         <v>11</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
+      <c r="A13" t="s" s="12">
+        <v>12</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
     </row>
     <row r="14">
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
+      <c r="A14" t="s" s="13">
+        <v>13</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
     </row>
     <row r="15">
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
+      <c r="A15" t="s" s="14">
+        <v>14</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
     </row>
     <row r="17">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
+      <c r="A17" s="20"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
@@ -579,7 +1109,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="s" s="5">
+      <c r="A152" t="s" s="15">
         <v>15</v>
       </c>
     </row>
@@ -589,7 +1119,7 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" t="s" s="7">
+      <c r="A252" t="s" s="17">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mejoras en generacion de examenes
</commit_message>
<xml_diff>
--- a/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
+++ b/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
   <si>
     <t>ALUMNO:</t>
   </si>
@@ -32,16 +32,10 @@
     <t>CONTENIDO 3:</t>
   </si>
   <si>
-    <t>CONTENIDO 4:</t>
-  </si>
-  <si>
-    <t>CONTENIDO 5:</t>
-  </si>
-  <si>
     <t>FECHA:</t>
   </si>
   <si>
-    <t>HORARIO</t>
+    <t>HORARIO:</t>
   </si>
   <si>
     <t>CORREO:</t>
@@ -59,16 +53,7 @@
     <t>PREGUNTA 3:</t>
   </si>
   <si>
-    <t>PREGUNTA 4:</t>
-  </si>
-  <si>
-    <t>PREGUNTA 5:</t>
-  </si>
-  <si>
-    <t>PREGUNTA 6:</t>
-  </si>
-  <si>
-    <t>ANDREA PERRINO</t>
+    <t>ALEJANDRO ARES</t>
   </si>
   <si>
     <t>1 BACHILLERATO</t>
@@ -78,21 +63,6 @@
   </si>
   <si>
     <t>Cinemática MRU MRUA MCU MCUA</t>
-  </si>
-  <si>
-    <t>Cinemática Tiro Parabólico</t>
-  </si>
-  <si>
-    <t>Cinemática Vectorial</t>
-  </si>
-  <si>
-    <t>Dinámica Cantidad Movimiento</t>
-  </si>
-  <si>
-    <t>Viernes, dia 14 de Agosto del 2026</t>
-  </si>
-  <si>
-    <t>A las: 16:00 horas</t>
   </si>
   <si>
     <t>CALIFICACIÓN</t>
@@ -103,7 +73,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="6">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -115,24 +85,6 @@
       <name val="Calibri"/>
       <sz val="11.0"/>
       <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -184,16 +136,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true"/>
   </cellXfs>
@@ -240,50 +189,12 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>97</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>2006600</xdr:colOff>
-      <xdr:row>99</xdr:row>
-      <xdr:rowOff>825500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="Picture"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2540000" cy="1206500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.0" customWidth="true"/>
@@ -295,10 +206,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="F1" t="s" s="8">
-        <v>27</v>
+        <v>13</v>
+      </c>
+      <c r="F1" t="s" s="5">
+        <v>17</v>
       </c>
     </row>
     <row r="2">
@@ -306,7 +217,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -314,31 +225,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
         <v>3</v>
       </c>
-      <c r="B4" t="s" s="0">
-        <v>21</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="1">
         <v>4</v>
       </c>
-      <c r="B5" t="s" s="0">
-        <v>22</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="1">
         <v>5</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -346,7 +251,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -354,7 +259,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -362,7 +267,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -370,84 +275,59 @@
         <v>9</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="1">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14">
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15">
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="17">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="3">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="4">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="5">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="s" s="6">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="s" s="7">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Terminado problema de la eleccion del numero preguntas
</commit_message>
<xml_diff>
--- a/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
+++ b/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>ALUMNO:</t>
   </si>
@@ -32,6 +32,12 @@
     <t>CONTENIDO 3:</t>
   </si>
   <si>
+    <t>CONTENIDO 4:</t>
+  </si>
+  <si>
+    <t>CONTENIDO 5:</t>
+  </si>
+  <si>
     <t>FECHA:</t>
   </si>
   <si>
@@ -53,16 +59,31 @@
     <t>PREGUNTA 3:</t>
   </si>
   <si>
+    <t>PREGUNTA 4:</t>
+  </si>
+  <si>
+    <t>PREGUNTA 5:</t>
+  </si>
+  <si>
+    <t>PREGUNTA 6:</t>
+  </si>
+  <si>
     <t>ALEJANDRO ARES</t>
   </si>
   <si>
     <t>1 BACHILLERATO</t>
   </si>
   <si>
-    <t>Física y Química</t>
-  </si>
-  <si>
-    <t>Cinemática MRU MRUA MCU MCUA</t>
+    <t>Dibujo Técnico</t>
+  </si>
+  <si>
+    <t>Construcción de Formas Polígonales</t>
+  </si>
+  <si>
+    <t>Jueves, dia 27 de Agosto del 2026</t>
+  </si>
+  <si>
+    <t>A las: 16:00 horas</t>
   </si>
   <si>
     <t>CALIFICACIÓN</t>
@@ -73,7 +94,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -85,6 +106,24 @@
       <name val="Calibri"/>
       <sz val="11.0"/>
       <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -136,13 +175,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true"/>
   </cellXfs>
@@ -189,12 +231,202 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>147</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>149</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>197</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>199</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>247</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>249</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>297</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2006600</xdr:colOff>
+      <xdr:row>299</xdr:row>
+      <xdr:rowOff>825500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 1" descr="Picture"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2540000" cy="1206500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H252"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.0" customWidth="true"/>
@@ -206,10 +438,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="F1" t="s" s="5">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="F1" t="s" s="8">
+        <v>24</v>
       </c>
     </row>
     <row r="2">
@@ -217,7 +449,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
@@ -225,25 +457,31 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
         <v>3</v>
       </c>
+      <c r="B4" t="s" s="0">
+        <v>21</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="1">
         <v>4</v>
       </c>
+      <c r="B5" t="s" s="0">
+        <v>21</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="1">
         <v>5</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -251,7 +489,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -259,7 +497,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -267,7 +505,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
@@ -275,59 +513,84 @@
         <v>9</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>16</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="1">
+        <v>11</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
     </row>
     <row r="14">
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
     </row>
     <row r="15">
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
     </row>
     <row r="17">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s" s="3">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="s" s="4">
         <v>12</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s" s="4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="s" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="s" s="6">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="s" s="7">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mejora en chat sockets
</commit_message>
<xml_diff>
--- a/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
+++ b/0001-Proyecto-Maven-POI/ficherosGenerados/examen.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>ALUMNO:</t>
   </si>
@@ -35,9 +35,6 @@
     <t>CONTENIDO 4:</t>
   </si>
   <si>
-    <t>CONTENIDO 5:</t>
-  </si>
-  <si>
     <t>FECHA:</t>
   </si>
   <si>
@@ -62,25 +59,28 @@
     <t>PREGUNTA 4:</t>
   </si>
   <si>
-    <t>PREGUNTA 5:</t>
-  </si>
-  <si>
-    <t>PREGUNTA 6:</t>
-  </si>
-  <si>
     <t>ALEJANDRO ARES</t>
   </si>
   <si>
-    <t>1 BACHILLERATO</t>
-  </si>
-  <si>
-    <t>Dibujo Técnico</t>
-  </si>
-  <si>
-    <t>Construcción de Formas Polígonales</t>
-  </si>
-  <si>
-    <t>Jueves, dia 27 de Agosto del 2026</t>
+    <t>2 BACHILLERATO</t>
+  </si>
+  <si>
+    <t>Física</t>
+  </si>
+  <si>
+    <t>Campo Eléctrico</t>
+  </si>
+  <si>
+    <t>Campo Gravitatorio</t>
+  </si>
+  <si>
+    <t>Campo Magnético</t>
+  </si>
+  <si>
+    <t>Física Moderna</t>
+  </si>
+  <si>
+    <t>Viernes, dia 28 de Agosto del 2026</t>
   </si>
   <si>
     <t>A las: 16:00 horas</t>
@@ -94,7 +94,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -106,18 +106,6 @@
       <name val="Calibri"/>
       <sz val="11.0"/>
       <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -175,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
@@ -183,8 +171,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true"/>
   </cellXfs>
@@ -269,164 +255,12 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>147</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>2006600</xdr:colOff>
-      <xdr:row>149</xdr:row>
-      <xdr:rowOff>825500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 1" descr="Picture"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2540000" cy="1206500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>197</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>2006600</xdr:colOff>
-      <xdr:row>199</xdr:row>
-      <xdr:rowOff>825500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 1" descr="Picture"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2540000" cy="1206500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>247</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>2006600</xdr:colOff>
-      <xdr:row>249</xdr:row>
-      <xdr:rowOff>825500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 1" descr="Picture"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2540000" cy="1206500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>297</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>2006600</xdr:colOff>
-      <xdr:row>299</xdr:row>
-      <xdr:rowOff>825500</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 1" descr="Picture"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2540000" cy="1206500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H252"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.0" customWidth="true"/>
@@ -438,9 +272,9 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="F1" t="s" s="8">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s" s="6">
         <v>24</v>
       </c>
     </row>
@@ -449,7 +283,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +291,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -465,7 +299,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -473,7 +307,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -481,7 +315,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +331,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -505,92 +339,74 @@
         <v>8</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="1">
         <v>9</v>
       </c>
-      <c r="B10" t="s" s="0">
-        <v>23</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="s" s="1">
-        <v>11</v>
-      </c>
-    </row>
     <row r="13">
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
     </row>
     <row r="14">
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
     </row>
     <row r="15">
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
     </row>
     <row r="17">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="3">
         <v>12</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="s" s="3">
+    <row r="39">
+      <c r="A39" t="s" s="4">
         <v>13</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" t="s" s="4">
+    <row r="51">
+      <c r="A51" t="s" s="5">
         <v>14</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="s" s="5">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="s" s="6">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="s" s="7">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>